<commit_message>
chore: run 2026-03-11 16:52 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_11_03_2026.xlsx
+++ b/logs/Consolidado_11_03_2026.xlsx
@@ -695,10 +695,10 @@
         <v>72</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -13582,12 +13582,12 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>8067425</t>
+          <t>8067439</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>3000716</t>
+          <t>3000714</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -13911,12 +13911,12 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>4468119</t>
+          <t>3000714</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -14869,40 +14869,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>11/03/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Color Glow Repairing Glow Conditioner
 Máscara Reparadora Cabelo Pintado e Madeixas
 200 ml</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/color-glow-repairing-glow-conditioner-7924433.html</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>7924433</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -15552,12 +15552,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>7610972</t>
+          <t>6633968</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -27406,12 +27406,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>8067425</t>
+          <t>8067439</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -27444,12 +27444,12 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>4468119</t>
+          <t>3000714</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -27482,7 +27482,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>3000716</t>
+          <t>3000714</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -27750,12 +27750,12 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>7610972</t>
+          <t>6633968</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-11 17:51 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_11_03_2026.xlsx
+++ b/logs/Consolidado_11_03_2026.xlsx
@@ -13868,7 +13868,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>3000714</t>
+          <t>3000716</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -13911,12 +13911,12 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>3000714</t>
+          <t>4468119</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -15552,12 +15552,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>6633968</t>
+          <t>7610972</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -27444,12 +27444,12 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>3000714</t>
+          <t>4468119</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -27482,7 +27482,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>3000714</t>
+          <t>3000716</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -27750,12 +27750,12 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>6633968</t>
+          <t>7610972</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-11 18:30 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_11_03_2026.xlsx
+++ b/logs/Consolidado_11_03_2026.xlsx
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>7106534</t>
+          <t>7106530</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -25319,7 +25319,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>7106534</t>
+          <t>7106530</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-11 20:17 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_11_03_2026.xlsx
+++ b/logs/Consolidado_11_03_2026.xlsx
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>7106530</t>
+          <t>7106534</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -15105,12 +15105,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>7630905</t>
+          <t>6759973</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -25319,7 +25319,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>7106530</t>
+          <t>7106534</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -27674,12 +27674,12 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>7630905</t>
+          <t>6759973</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-03-11 21:46 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_11_03_2026.xlsx
+++ b/logs/Consolidado_11_03_2026.xlsx
@@ -657,10 +657,10 @@
         <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -676,10 +676,10 @@
         <v>82</v>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -9963,40 +9963,40 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>11/03/2026</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>Sensinol Shampooing Physioprotecteur
 Champô Calmante Couro Cabeludo Sensível
 400 ml</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/sensinol-shampooing-physioprotecteur-7646502.html</t>
         </is>
       </c>
-      <c r="E67" s="3" t="inlineStr"/>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
         <is>
           <t>7646502</t>
         </is>
       </c>
-      <c r="H67" s="3" t="inlineStr">
+      <c r="H67" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -12879,43 +12879,43 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>11/03/2026</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>Nettle &amp; Vitamin E Oil Control Dry Shampoo
 Champô Seco Ortiga BIO Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-and-vitamin-e-oil-control-dry-shampoo-366180.html</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E66" s="7" t="inlineStr">
         <is>
           <t>150 ml</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>8123759</t>
         </is>
       </c>
-      <c r="H66" s="5" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -15105,12 +15105,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>6759973</t>
+          <t>7630905</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -26965,38 +26965,38 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>Nettle &amp; Vitamin E Oil Control Dry Shampoo
 Champô Seco Ortiga BIO Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>150 ml</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>8123759</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-and-vitamin-e-oil-control-dry-shampoo-366180.html</t>
         </is>
@@ -27674,12 +27674,12 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>6759973</t>
+          <t>7630905</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">

</xml_diff>